<commit_message>
Add Critically Acclaimed video (Vimeo 1216821430) to videos.xlsx
</commit_message>
<xml_diff>
--- a/videos.xlsx
+++ b/videos.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Videos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Videos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -660,6 +660,18 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1216821430?share=copy&amp;fl=sv&amp;fe=ci</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Critically Acclaimed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove Vimeo 1216821430 from videos.xlsx
</commit_message>
<xml_diff>
--- a/videos.xlsx
+++ b/videos.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -660,18 +660,6 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>https://vimeo.com/1216821430?share=copy&amp;fl=sv&amp;fe=ci</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Critically Acclaimed</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove Spooky Slime video (Vimeo 1216821504) from videos.xlsx
</commit_message>
<xml_diff>
--- a/videos.xlsx
+++ b/videos.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -598,7 +598,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1216821504</t>
+          <t>https://vimeo.com/1216821503</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -610,51 +610,39 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1216821503</t>
+          <t>https://vimeo.com/1216712429</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Segments &amp; Highlights</t>
+          <t>Archives</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1216712429</t>
+          <t>https://vimeo.com/1216712427</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>Archives</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>TRUE</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1216712427</t>
+          <t>https://vimeo.com/1216821487</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
-        <is>
-          <t>Archives</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>https://vimeo.com/1216821487</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
         <is>
           <t>Archives</t>
         </is>

</xml_diff>